<commit_message>
v0.4.0: Add data catalog, suspicious match detection, PRD, and README
- Data catalog (207 stats across team/player/derived categories)
- Score-based forfeit detection (32 invalid matches identified)
- Product requirements document for broadcast stats dashboard
- README with version history and project overview

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FOKUS_Stats.xlsx
+++ b/FOKUS_Stats.xlsx
@@ -180,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,7 +226,16 @@
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -241,16 +250,16 @@
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1979,7 +1988,7 @@
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="10" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>11</v>
@@ -1994,10 +2003,10 @@
         <v>0.547085201793722</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>0.5390625</v>
+        <v>0.5433070866141733</v>
       </c>
       <c r="O7" s="11" t="n">
-        <v>0.5578947368421052</v>
+        <v>0.5520833333333334</v>
       </c>
       <c r="P7" s="11" t="n">
         <v>0.4545454545454545</v>
@@ -2012,10 +2021,10 @@
         <v>0.6024096385542169</v>
       </c>
       <c r="T7" s="13" t="n">
-        <v>0.6122448979591837</v>
+        <v>0.6185567010309279</v>
       </c>
       <c r="U7" s="11" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.5797101449275363</v>
       </c>
       <c r="V7" s="11" t="n">
         <v>0.5</v>
@@ -2044,7 +2053,7 @@
         <v>93</v>
       </c>
       <c r="AF7" s="10" t="n">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="AG7" s="10" t="n">
         <v>8.449999999999999</v>
@@ -2057,7 +2066,7 @@
         <v>67</v>
       </c>
       <c r="AK7" s="10" t="n">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="AL7" s="10" t="n">
         <v>6.09</v>
@@ -2101,10 +2110,10 @@
         <v>0.6187845303867403</v>
       </c>
       <c r="N8" s="18" t="n">
-        <v>0.504950495049505</v>
+        <v>0.5098039215686274</v>
       </c>
       <c r="O8" s="17" t="n">
-        <v>0.7625</v>
+        <v>0.759493670886076</v>
       </c>
       <c r="P8" s="18" t="n">
         <v>0.5</v>
@@ -2119,10 +2128,10 @@
         <v>0.6838235294117647</v>
       </c>
       <c r="T8" s="18" t="n">
-        <v>0.5921052631578947</v>
+        <v>0.5974025974025974</v>
       </c>
       <c r="U8" s="17" t="n">
-        <v>0.8</v>
+        <v>0.7966101694915254</v>
       </c>
       <c r="V8" s="18" t="n">
         <v>0.4444444444444444</v>
@@ -2147,7 +2156,7 @@
         <v>69</v>
       </c>
       <c r="AF8" s="16" t="n">
-        <v>68</v>
+        <v>102</v>
       </c>
       <c r="AG8" s="16" t="n">
         <v>7.67</v>
@@ -2160,7 +2169,7 @@
         <v>47</v>
       </c>
       <c r="AK8" s="16" t="n">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="AL8" s="16" t="n">
         <v>5.22</v>
@@ -2189,7 +2198,7 @@
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="6" t="n"/>
       <c r="I9" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>8</v>
@@ -2204,10 +2213,10 @@
         <v>0.5480225988700564</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>0.5869565217391305</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>0.5058823529411764</v>
+        <v>0.5232558139534884</v>
       </c>
       <c r="P9" s="12" t="n">
         <v>0.375</v>
@@ -2222,10 +2231,10 @@
         <v>0.5755395683453237</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>0.6351351351351351</v>
+        <v>0.6164383561643836</v>
       </c>
       <c r="U9" s="11" t="n">
-        <v>0.5076923076923077</v>
+        <v>0.5303030303030303</v>
       </c>
       <c r="V9" s="11" t="n">
         <v>0.5625</v>
@@ -2250,7 +2259,7 @@
         <v>70</v>
       </c>
       <c r="AF9" s="10" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="AG9" s="10" t="n">
         <v>8.75</v>
@@ -2263,7 +2272,7 @@
         <v>54</v>
       </c>
       <c r="AK9" s="10" t="n">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="AL9" s="10" t="n">
         <v>6.75</v>
@@ -2292,7 +2301,7 @@
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="16" t="n">
         <v>6</v>
@@ -2357,7 +2366,7 @@
         <v>49</v>
       </c>
       <c r="AF10" s="16" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="AG10" s="16" t="n">
         <v>8.17</v>
@@ -2370,7 +2379,7 @@
         <v>32</v>
       </c>
       <c r="AK10" s="16" t="n">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="AL10" s="16" t="n">
         <v>5.33</v>
@@ -2399,7 +2408,7 @@
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>7</v>
@@ -2464,7 +2473,7 @@
         <v>45</v>
       </c>
       <c r="AF11" s="10" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="AG11" s="10" t="n">
         <v>6.43</v>
@@ -2477,7 +2486,7 @@
         <v>56</v>
       </c>
       <c r="AK11" s="10" t="n">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="AL11" s="10" t="n">
         <v>8</v>
@@ -2567,7 +2576,7 @@
         <v>20</v>
       </c>
       <c r="AF12" s="16" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AG12" s="16" t="n">
         <v>10</v>
@@ -2580,7 +2589,7 @@
         <v>16</v>
       </c>
       <c r="AK12" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AL12" s="16" t="n">
         <v>8</v>
@@ -2609,7 +2618,7 @@
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>6</v>
@@ -2674,7 +2683,7 @@
         <v>33</v>
       </c>
       <c r="AF13" s="10" t="n">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="AG13" s="10" t="n">
         <v>5.5</v>
@@ -2687,7 +2696,7 @@
         <v>33</v>
       </c>
       <c r="AK13" s="10" t="n">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="AL13" s="10" t="n">
         <v>5.5</v>
@@ -2727,10 +2736,10 @@
         <v>0.5731462925851704</v>
       </c>
       <c r="N14" s="21" t="n">
-        <v>0.5738963531669866</v>
+        <v>0.573076923076923</v>
       </c>
       <c r="O14" s="21" t="n">
-        <v>0.5723270440251572</v>
+        <v>0.5732217573221757</v>
       </c>
       <c r="P14" s="21" t="n">
         <v>0.5204081632653061</v>
@@ -2745,10 +2754,10 @@
         <v>0.6114819759679573</v>
       </c>
       <c r="T14" s="22" t="n">
-        <v>0.6080402010050251</v>
+        <v>0.6070528967254408</v>
       </c>
       <c r="U14" s="22" t="n">
-        <v>0.6153846153846154</v>
+        <v>0.6164772727272727</v>
       </c>
       <c r="V14" s="21" t="n">
         <v>0.5204081632653061</v>
@@ -2779,7 +2788,7 @@
         <v>379</v>
       </c>
       <c r="AF14" s="7" t="n">
-        <v>378</v>
+        <v>520</v>
       </c>
       <c r="AG14" s="7" t="n">
         <v>7.73</v>
@@ -2792,7 +2801,7 @@
         <v>305</v>
       </c>
       <c r="AK14" s="7" t="n">
-        <v>303</v>
+        <v>478</v>
       </c>
       <c r="AL14" s="7" t="n">
         <v>6.22</v>
@@ -2910,18 +2919,18 @@
       <c r="N17" s="5" t="n"/>
       <c r="O17" s="6" t="n"/>
       <c r="P17" s="1" t="n"/>
-      <c r="Q17" s="4" t="inlineStr">
+      <c r="Q17" s="1" t="n"/>
+      <c r="R17" s="1" t="n"/>
+      <c r="S17" s="4" t="inlineStr">
         <is>
           <t>Team XvY</t>
         </is>
       </c>
-      <c r="R17" s="5" t="n"/>
-      <c r="S17" s="5" t="n"/>
       <c r="T17" s="5" t="n"/>
       <c r="U17" s="5" t="n"/>
-      <c r="V17" s="6" t="n"/>
-      <c r="W17" s="1" t="n"/>
-      <c r="X17" s="1" t="n"/>
+      <c r="V17" s="5" t="n"/>
+      <c r="W17" s="5" t="n"/>
+      <c r="X17" s="6" t="n"/>
       <c r="Y17" s="1" t="n"/>
       <c r="Z17" s="1" t="n"/>
       <c r="AA17" s="1" t="n"/>
@@ -2999,36 +3008,40 @@
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
+          <t>AWP%</t>
+        </is>
+      </c>
+      <c r="R18" s="1" t="n"/>
+      <c r="S18" s="7" t="inlineStr">
+        <is>
           <t>X v Y</t>
         </is>
       </c>
-      <c r="R18" s="7" t="inlineStr">
+      <c r="T18" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="S18" s="7" t="inlineStr">
+      <c r="U18" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="T18" s="7" t="inlineStr">
+      <c r="V18" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="U18" s="7" t="inlineStr">
+      <c r="W18" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="V18" s="7" t="inlineStr">
+      <c r="X18" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="W18" s="1" t="n"/>
-      <c r="X18" s="1" t="n"/>
       <c r="Y18" s="1" t="n"/>
       <c r="Z18" s="1" t="n"/>
       <c r="AA18" s="1" t="n"/>
@@ -3090,20 +3103,30 @@
       <c r="P19" s="28" t="n">
         <v>0.1769911504424779</v>
       </c>
-      <c r="Q19" s="29" t="inlineStr">
+      <c r="Q19" s="29" t="n">
+        <v>0.1045340050377834</v>
+      </c>
+      <c r="R19" s="1" t="n"/>
+      <c r="S19" s="30" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="R19" s="1" t="n"/>
-      <c r="S19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="1" t="n"/>
-      <c r="U19" s="1" t="n"/>
-      <c r="V19" s="1" t="n"/>
-      <c r="W19" s="1" t="n"/>
-      <c r="X19" s="1" t="n"/>
+      <c r="T19" s="31" t="n">
+        <v>0.5731462925851704</v>
+      </c>
+      <c r="U19" s="31" t="n">
+        <v>0.7702205882352942</v>
+      </c>
+      <c r="V19" s="32" t="n">
+        <v>0.9392857142857143</v>
+      </c>
+      <c r="W19" s="32" t="n">
+        <v>0.9823529411764705</v>
+      </c>
+      <c r="X19" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="Y19" s="1" t="n"/>
       <c r="Z19" s="1" t="n"/>
       <c r="AA19" s="1" t="n"/>
@@ -3142,13 +3165,13 @@
       <c r="I20" s="16" t="n">
         <v>998</v>
       </c>
-      <c r="J20" s="30" t="n">
+      <c r="J20" s="33" t="n">
         <v>1.18</v>
       </c>
-      <c r="K20" s="30" t="n">
+      <c r="K20" s="33" t="n">
         <v>1.48</v>
       </c>
-      <c r="L20" s="31" t="n">
+      <c r="L20" s="34" t="n">
         <v>0.717434869739479</v>
       </c>
       <c r="M20" s="16" t="n">
@@ -3157,30 +3180,38 @@
       <c r="N20" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="O20" s="32" t="inlineStr">
+      <c r="O20" s="35" t="inlineStr">
         <is>
           <t>55%</t>
         </is>
       </c>
-      <c r="P20" s="33" t="n">
+      <c r="P20" s="36" t="n">
         <v>0.141025641025641</v>
       </c>
-      <c r="Q20" s="34" t="inlineStr">
+      <c r="Q20" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="1" t="n"/>
+      <c r="S20" s="38" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="R20" s="35" t="n">
+      <c r="T20" s="39" t="n">
+        <v>0.3370044052863436</v>
+      </c>
+      <c r="U20" s="39" t="n">
         <v>0.5636363636363636</v>
       </c>
-      <c r="S20" s="16" t="n">
-        <v>495</v>
-      </c>
-      <c r="T20" s="1" t="n"/>
-      <c r="U20" s="1" t="n"/>
-      <c r="V20" s="1" t="n"/>
-      <c r="W20" s="1" t="n"/>
-      <c r="X20" s="1" t="n"/>
+      <c r="V20" s="40" t="n">
+        <v>0.8063660477453581</v>
+      </c>
+      <c r="W20" s="40" t="n">
+        <v>0.9357142857142857</v>
+      </c>
+      <c r="X20" s="40" t="n">
+        <v>0.995049504950495</v>
+      </c>
       <c r="Y20" s="1" t="n"/>
       <c r="Z20" s="1" t="n"/>
       <c r="AA20" s="1" t="n"/>
@@ -3242,22 +3273,30 @@
       <c r="P21" s="28" t="n">
         <v>0.1240875912408759</v>
       </c>
-      <c r="Q21" s="29" t="inlineStr">
+      <c r="Q21" s="29" t="n">
+        <v>0.002941176470588235</v>
+      </c>
+      <c r="R21" s="1" t="n"/>
+      <c r="S21" s="30" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="R21" s="36" t="n">
-        <v>0.6388888888888888</v>
-      </c>
-      <c r="S21" s="10" t="n">
-        <v>72</v>
-      </c>
-      <c r="T21" s="1" t="n"/>
-      <c r="U21" s="1" t="n"/>
-      <c r="V21" s="1" t="n"/>
-      <c r="W21" s="1" t="n"/>
-      <c r="X21" s="1" t="n"/>
+      <c r="T21" s="28" t="n">
+        <v>0.1345291479820628</v>
+      </c>
+      <c r="U21" s="31" t="n">
+        <v>0.2852852852852853</v>
+      </c>
+      <c r="V21" s="31" t="n">
+        <v>0.5862068965517241</v>
+      </c>
+      <c r="W21" s="32" t="n">
+        <v>0.802013422818792</v>
+      </c>
+      <c r="X21" s="32" t="n">
+        <v>0.970954356846473</v>
+      </c>
       <c r="Y21" s="1" t="n"/>
       <c r="Z21" s="1" t="n"/>
       <c r="AA21" s="1" t="n"/>
@@ -3296,13 +3335,13 @@
       <c r="I22" s="16" t="n">
         <v>998</v>
       </c>
-      <c r="J22" s="30" t="n">
+      <c r="J22" s="33" t="n">
         <v>1.15</v>
       </c>
-      <c r="K22" s="30" t="n">
+      <c r="K22" s="33" t="n">
         <v>1.4</v>
       </c>
-      <c r="L22" s="31" t="n">
+      <c r="L22" s="34" t="n">
         <v>0.7104208416833667</v>
       </c>
       <c r="M22" s="16" t="n">
@@ -3311,30 +3350,38 @@
       <c r="N22" s="16" t="n">
         <v>0.17</v>
       </c>
-      <c r="O22" s="32" t="inlineStr">
+      <c r="O22" s="35" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="P22" s="35" t="n">
+      <c r="P22" s="39" t="n">
         <v>0.2608695652173913</v>
       </c>
-      <c r="Q22" s="34" t="inlineStr">
+      <c r="Q22" s="37" t="n">
+        <v>0.02545454545454546</v>
+      </c>
+      <c r="R22" s="1" t="n"/>
+      <c r="S22" s="38" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="R22" s="35" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="S22" s="16" t="n">
-        <v>36</v>
-      </c>
-      <c r="T22" s="1" t="n"/>
-      <c r="U22" s="1" t="n"/>
-      <c r="V22" s="1" t="n"/>
-      <c r="W22" s="1" t="n"/>
-      <c r="X22" s="1" t="n"/>
+      <c r="T22" s="36" t="n">
+        <v>0.02631578947368421</v>
+      </c>
+      <c r="U22" s="36" t="n">
+        <v>0.0752212389380531</v>
+      </c>
+      <c r="V22" s="39" t="n">
+        <v>0.2554112554112554</v>
+      </c>
+      <c r="W22" s="39" t="n">
+        <v>0.5324675324675324</v>
+      </c>
+      <c r="X22" s="40" t="n">
+        <v>0.883495145631068</v>
+      </c>
       <c r="Y22" s="1" t="n"/>
       <c r="Z22" s="1" t="n"/>
       <c r="AA22" s="1" t="n"/>
@@ -3396,22 +3443,30 @@
       <c r="P23" s="28" t="n">
         <v>0.1376146788990826</v>
       </c>
-      <c r="Q23" s="29" t="inlineStr">
+      <c r="Q23" s="29" t="n">
+        <v>0.001538461538461538</v>
+      </c>
+      <c r="R23" s="1" t="n"/>
+      <c r="S23" s="30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R23" s="37" t="n">
+      <c r="T23" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="28" t="n">
+        <v>0.02013422818791946</v>
+      </c>
+      <c r="V23" s="28" t="n">
+        <v>0.05978260869565218</v>
+      </c>
+      <c r="W23" s="28" t="n">
+        <v>0.1602209944751381</v>
+      </c>
+      <c r="X23" s="31" t="n">
         <v>0.5</v>
       </c>
-      <c r="S23" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="T23" s="1" t="n"/>
-      <c r="U23" s="1" t="n"/>
-      <c r="V23" s="1" t="n"/>
-      <c r="W23" s="1" t="n"/>
-      <c r="X23" s="1" t="n"/>
       <c r="Y23" s="1" t="n"/>
       <c r="Z23" s="1" t="n"/>
       <c r="AA23" s="1" t="n"/>
@@ -4345,7 +4400,6 @@
     <mergeCell ref="AJ5:AO5"/>
     <mergeCell ref="D11:H11"/>
     <mergeCell ref="D13:H13"/>
-    <mergeCell ref="Q17:V17"/>
     <mergeCell ref="D7:H7"/>
     <mergeCell ref="S5:U5"/>
     <mergeCell ref="P5:R5"/>
@@ -4360,6 +4414,7 @@
     <mergeCell ref="AD5:AI5"/>
     <mergeCell ref="M5:O5"/>
     <mergeCell ref="D23:H23"/>
+    <mergeCell ref="S17:X17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4441,12 +4496,12 @@
       <c r="E2" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F2" s="38" t="inlineStr">
+      <c r="F2" s="41" t="inlineStr">
         <is>
           <t>adf2c80a-a27b-433b-943b-05f278d63913</t>
         </is>
       </c>
-      <c r="G2" s="39" t="inlineStr">
+      <c r="G2" s="42" t="inlineStr">
         <is>
           <t>Tech issue / forfeit</t>
         </is>
@@ -4474,12 +4529,12 @@
       <c r="E3" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F3" s="40" t="inlineStr">
+      <c r="F3" s="43" t="inlineStr">
         <is>
           <t>b488c914-49ec-41c2-afcb-e76a8696d6dd</t>
         </is>
       </c>
-      <c r="G3" s="41" t="inlineStr">
+      <c r="G3" s="44" t="inlineStr">
         <is>
           <t>Tech issue / forfeit</t>
         </is>
@@ -4507,61 +4562,61 @@
       <c r="E4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="38" t="inlineStr">
+      <c r="F4" s="41" t="inlineStr">
         <is>
           <t>f973d754-9985-498f-bcca-79499822a699</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="42" t="inlineStr">
         <is>
           <t>Tech issue / forfeit</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="42" t="n"/>
-      <c r="B5" s="42" t="n"/>
-      <c r="C5" s="42" t="n"/>
-      <c r="D5" s="42" t="n"/>
-      <c r="E5" s="42" t="n"/>
-      <c r="F5" s="42" t="n"/>
-      <c r="G5" s="42" t="n"/>
+      <c r="A5" s="45" t="n"/>
+      <c r="B5" s="45" t="n"/>
+      <c r="C5" s="45" t="n"/>
+      <c r="D5" s="45" t="n"/>
+      <c r="E5" s="45" t="n"/>
+      <c r="F5" s="45" t="n"/>
+      <c r="G5" s="45" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="42" t="n"/>
-      <c r="B6" s="42" t="n"/>
-      <c r="C6" s="42" t="n"/>
-      <c r="D6" s="42" t="n"/>
-      <c r="E6" s="42" t="n"/>
-      <c r="F6" s="42" t="n"/>
-      <c r="G6" s="42" t="n"/>
+      <c r="A6" s="45" t="n"/>
+      <c r="B6" s="45" t="n"/>
+      <c r="C6" s="45" t="n"/>
+      <c r="D6" s="45" t="n"/>
+      <c r="E6" s="45" t="n"/>
+      <c r="F6" s="45" t="n"/>
+      <c r="G6" s="45" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="42" t="n"/>
-      <c r="B7" s="42" t="n"/>
-      <c r="C7" s="42" t="n"/>
-      <c r="D7" s="42" t="n"/>
-      <c r="E7" s="42" t="n"/>
-      <c r="F7" s="42" t="n"/>
-      <c r="G7" s="42" t="n"/>
+      <c r="A7" s="45" t="n"/>
+      <c r="B7" s="45" t="n"/>
+      <c r="C7" s="45" t="n"/>
+      <c r="D7" s="45" t="n"/>
+      <c r="E7" s="45" t="n"/>
+      <c r="F7" s="45" t="n"/>
+      <c r="G7" s="45" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="42" t="n"/>
-      <c r="B8" s="42" t="n"/>
-      <c r="C8" s="42" t="n"/>
-      <c r="D8" s="42" t="n"/>
-      <c r="E8" s="42" t="n"/>
-      <c r="F8" s="42" t="n"/>
-      <c r="G8" s="42" t="n"/>
+      <c r="A8" s="45" t="n"/>
+      <c r="B8" s="45" t="n"/>
+      <c r="C8" s="45" t="n"/>
+      <c r="D8" s="45" t="n"/>
+      <c r="E8" s="45" t="n"/>
+      <c r="F8" s="45" t="n"/>
+      <c r="G8" s="45" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="42" t="n"/>
-      <c r="B9" s="42" t="n"/>
-      <c r="C9" s="42" t="n"/>
-      <c r="D9" s="42" t="n"/>
-      <c r="E9" s="42" t="n"/>
-      <c r="F9" s="42" t="n"/>
-      <c r="G9" s="42" t="n"/>
+      <c r="A9" s="45" t="n"/>
+      <c r="B9" s="45" t="n"/>
+      <c r="C9" s="45" t="n"/>
+      <c r="D9" s="45" t="n"/>
+      <c r="E9" s="45" t="n"/>
+      <c r="F9" s="45" t="n"/>
+      <c r="G9" s="45" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4647,7 +4702,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G2" s="38" t="inlineStr">
+      <c r="G2" s="41" t="inlineStr">
         <is>
           <t>99540cbf-5ce1-468a-a75b-cad599a066f1</t>
         </is>
@@ -4675,12 +4730,12 @@
       <c r="E3" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="30" t="inlineStr">
+      <c r="F3" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G3" s="40" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t>3b4f89bd-5eb9-4514-afc0-999106e723ef</t>
         </is>
@@ -4708,12 +4763,12 @@
       <c r="E4" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F4" s="43" t="inlineStr">
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G4" s="38" t="inlineStr">
+      <c r="G4" s="41" t="inlineStr">
         <is>
           <t>251458f5-e226-4f91-9105-495585aa6e4e</t>
         </is>
@@ -4741,12 +4796,12 @@
       <c r="E5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="30" t="inlineStr">
+      <c r="F5" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G5" s="40" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t>d47a35b8-c62e-4edc-b7f5-a38f12a06375</t>
         </is>
@@ -4779,7 +4834,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G6" s="38" t="inlineStr">
+      <c r="G6" s="41" t="inlineStr">
         <is>
           <t>63ef3ce4-bed1-49da-b13b-8d80756f98bb</t>
         </is>
@@ -4807,12 +4862,12 @@
       <c r="E7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="30" t="inlineStr">
+      <c r="F7" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G7" s="40" t="inlineStr">
+      <c r="G7" s="43" t="inlineStr">
         <is>
           <t>f146170a-8980-4544-93ec-8ad473392e2d</t>
         </is>
@@ -4845,7 +4900,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G8" s="38" t="inlineStr">
+      <c r="G8" s="41" t="inlineStr">
         <is>
           <t>c2d26138-4ee8-4c0e-9250-9ddedf9e300b</t>
         </is>
@@ -4873,12 +4928,12 @@
       <c r="E9" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F9" s="44" t="inlineStr">
+      <c r="F9" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G9" s="40" t="inlineStr">
+      <c r="G9" s="43" t="inlineStr">
         <is>
           <t>026f5435-c303-4f77-be11-be97b0add9fc</t>
         </is>
@@ -4911,7 +4966,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G10" s="38" t="inlineStr">
+      <c r="G10" s="41" t="inlineStr">
         <is>
           <t>168a93e8-447f-4216-9aad-b32dd36ac14f</t>
         </is>
@@ -4939,12 +4994,12 @@
       <c r="E11" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F11" s="30" t="inlineStr">
+      <c r="F11" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G11" s="40" t="inlineStr">
+      <c r="G11" s="43" t="inlineStr">
         <is>
           <t>3f27c0e4-1519-4462-951a-c92320aa226b</t>
         </is>
@@ -4977,7 +5032,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G12" s="38" t="inlineStr">
+      <c r="G12" s="41" t="inlineStr">
         <is>
           <t>11e2b172-f543-47dc-8b37-f1d25b6fce87</t>
         </is>
@@ -5005,12 +5060,12 @@
       <c r="E13" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F13" s="30" t="inlineStr">
+      <c r="F13" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G13" s="40" t="inlineStr">
+      <c r="G13" s="43" t="inlineStr">
         <is>
           <t>5ca51915-1449-471b-821d-b5cfc8cc5cb5</t>
         </is>
@@ -5043,7 +5098,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G14" s="38" t="inlineStr">
+      <c r="G14" s="41" t="inlineStr">
         <is>
           <t>cea3d447-0e22-4414-93cd-6b7e1d0d340a</t>
         </is>
@@ -5071,12 +5126,12 @@
       <c r="E15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="30" t="inlineStr">
+      <c r="F15" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G15" s="40" t="inlineStr">
+      <c r="G15" s="43" t="inlineStr">
         <is>
           <t>a1bd7228-1020-49ca-a3a1-51a7e376cfb2</t>
         </is>
@@ -5109,7 +5164,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G16" s="38" t="inlineStr">
+      <c r="G16" s="41" t="inlineStr">
         <is>
           <t>71a412d1-d670-429c-b022-77c9c007fae6</t>
         </is>
@@ -5137,12 +5192,12 @@
       <c r="E17" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F17" s="30" t="inlineStr">
+      <c r="F17" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G17" s="40" t="inlineStr">
+      <c r="G17" s="43" t="inlineStr">
         <is>
           <t>4f384665-abc0-4d4e-a46a-1295fa024c96</t>
         </is>
@@ -5175,7 +5230,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G18" s="38" t="inlineStr">
+      <c r="G18" s="41" t="inlineStr">
         <is>
           <t>44af6d79-4f89-4504-81a4-cf5812821245</t>
         </is>
@@ -5203,12 +5258,12 @@
       <c r="E19" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="30" t="inlineStr">
+      <c r="F19" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G19" s="40" t="inlineStr">
+      <c r="G19" s="43" t="inlineStr">
         <is>
           <t>dc4e1fa3-98e3-4d15-96fc-a1dbbf639ad2</t>
         </is>
@@ -5241,7 +5296,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G20" s="38" t="inlineStr">
+      <c r="G20" s="41" t="inlineStr">
         <is>
           <t>225cb9d4-7df5-40c4-8d62-ab3253b5bccd</t>
         </is>
@@ -5269,12 +5324,12 @@
       <c r="E21" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F21" s="30" t="inlineStr">
+      <c r="F21" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G21" s="40" t="inlineStr">
+      <c r="G21" s="43" t="inlineStr">
         <is>
           <t>8abc3599-746b-489a-ab51-e8dd2da1f2ee</t>
         </is>
@@ -5307,7 +5362,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G22" s="38" t="inlineStr">
+      <c r="G22" s="41" t="inlineStr">
         <is>
           <t>346d5ff3-a10d-4282-b076-c14bbf762d01</t>
         </is>
@@ -5335,12 +5390,12 @@
       <c r="E23" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="30" t="inlineStr">
+      <c r="F23" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G23" s="40" t="inlineStr">
+      <c r="G23" s="43" t="inlineStr">
         <is>
           <t>b39fd1eb-97b2-41f4-998d-a24649106a4d</t>
         </is>
@@ -5368,12 +5423,12 @@
       <c r="E24" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F24" s="43" t="inlineStr">
+      <c r="F24" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G24" s="38" t="inlineStr">
+      <c r="G24" s="41" t="inlineStr">
         <is>
           <t>f3736b8c-af86-4c9a-9906-9ca7eaa1c4ed</t>
         </is>
@@ -5401,12 +5456,12 @@
       <c r="E25" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="F25" s="44" t="inlineStr">
+      <c r="F25" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G25" s="40" t="inlineStr">
+      <c r="G25" s="43" t="inlineStr">
         <is>
           <t>0a248793-a692-4c20-8be9-7c0bd9e056ea</t>
         </is>
@@ -5434,12 +5489,12 @@
       <c r="E26" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F26" s="43" t="inlineStr">
+      <c r="F26" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G26" s="38" t="inlineStr">
+      <c r="G26" s="41" t="inlineStr">
         <is>
           <t>dada73b7-50c6-4330-958e-8cbbfb175634</t>
         </is>
@@ -5467,12 +5522,12 @@
       <c r="E27" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="F27" s="30" t="inlineStr">
+      <c r="F27" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G27" s="40" t="inlineStr">
+      <c r="G27" s="43" t="inlineStr">
         <is>
           <t>efb962fe-8292-4b05-8113-4a8f79fa5a8b</t>
         </is>
@@ -5505,7 +5560,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G28" s="38" t="inlineStr">
+      <c r="G28" s="41" t="inlineStr">
         <is>
           <t>8cf2bdd2-6e4a-483c-ba68-109f21f7d47a</t>
         </is>
@@ -5533,12 +5588,12 @@
       <c r="E29" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F29" s="44" t="inlineStr">
+      <c r="F29" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G29" s="40" t="inlineStr">
+      <c r="G29" s="43" t="inlineStr">
         <is>
           <t>c7c1710e-25af-4247-83c9-6184f561abc9</t>
         </is>
@@ -5571,7 +5626,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G30" s="38" t="inlineStr">
+      <c r="G30" s="41" t="inlineStr">
         <is>
           <t>0b839669-3599-4397-b854-cfa50df59d32</t>
         </is>
@@ -5599,12 +5654,12 @@
       <c r="E31" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F31" s="44" t="inlineStr">
+      <c r="F31" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G31" s="40" t="inlineStr">
+      <c r="G31" s="43" t="inlineStr">
         <is>
           <t>d9061177-8c07-4b8a-933c-09d671580f04</t>
         </is>
@@ -5632,12 +5687,12 @@
       <c r="E32" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F32" s="43" t="inlineStr">
+      <c r="F32" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G32" s="38" t="inlineStr">
+      <c r="G32" s="41" t="inlineStr">
         <is>
           <t>b1b2498b-0fa9-483b-a9f0-362d3f4b2f08</t>
         </is>
@@ -5665,12 +5720,12 @@
       <c r="E33" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F33" s="44" t="inlineStr">
+      <c r="F33" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G33" s="40" t="inlineStr">
+      <c r="G33" s="43" t="inlineStr">
         <is>
           <t>23790ccf-906d-4357-9360-76c4bef175b7</t>
         </is>
@@ -5698,12 +5753,12 @@
       <c r="E34" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F34" s="43" t="inlineStr">
+      <c r="F34" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G34" s="38" t="inlineStr">
+      <c r="G34" s="41" t="inlineStr">
         <is>
           <t>d94fe112-5977-4c0e-9bf7-65fc004dc43f</t>
         </is>
@@ -5731,12 +5786,12 @@
       <c r="E35" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F35" s="30" t="inlineStr">
+      <c r="F35" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G35" s="40" t="inlineStr">
+      <c r="G35" s="43" t="inlineStr">
         <is>
           <t>e7082892-d52a-4fa2-bfe0-16d74f4ff0d1</t>
         </is>
@@ -5764,12 +5819,12 @@
       <c r="E36" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F36" s="43" t="inlineStr">
+      <c r="F36" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G36" s="38" t="inlineStr">
+      <c r="G36" s="41" t="inlineStr">
         <is>
           <t>b18cf372-aa87-4cde-9167-061914581c8e</t>
         </is>
@@ -5797,12 +5852,12 @@
       <c r="E37" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F37" s="44" t="inlineStr">
+      <c r="F37" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G37" s="40" t="inlineStr">
+      <c r="G37" s="43" t="inlineStr">
         <is>
           <t>9cc27d5c-07e0-460c-be48-434902f91cc3</t>
         </is>
@@ -5835,7 +5890,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G38" s="38" t="inlineStr">
+      <c r="G38" s="41" t="inlineStr">
         <is>
           <t>1c3f1cc3-056e-44ea-b9a4-56a817fd7829</t>
         </is>
@@ -5863,12 +5918,12 @@
       <c r="E39" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="F39" s="30" t="inlineStr">
+      <c r="F39" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G39" s="40" t="inlineStr">
+      <c r="G39" s="43" t="inlineStr">
         <is>
           <t>01a75b22-a80e-4438-b648-bdc89fe6f0bb</t>
         </is>
@@ -5901,7 +5956,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G40" s="38" t="inlineStr">
+      <c r="G40" s="41" t="inlineStr">
         <is>
           <t>83cd5fda-a318-4ab6-b814-354737fa43e3</t>
         </is>
@@ -5929,12 +5984,12 @@
       <c r="E41" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F41" s="30" t="inlineStr">
+      <c r="F41" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G41" s="40" t="inlineStr">
+      <c r="G41" s="43" t="inlineStr">
         <is>
           <t>8772c4f9-8c25-46b6-ace7-4625e7fad180</t>
         </is>
@@ -5967,7 +6022,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G42" s="38" t="inlineStr">
+      <c r="G42" s="41" t="inlineStr">
         <is>
           <t>a9d924dd-7d4c-497c-91cb-1b22234d4e0d</t>
         </is>
@@ -5995,12 +6050,12 @@
       <c r="E43" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F43" s="44" t="inlineStr">
+      <c r="F43" s="47" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G43" s="40" t="inlineStr">
+      <c r="G43" s="43" t="inlineStr">
         <is>
           <t>8a58d3fb-4ee0-4cbc-b09a-93ce5733c2b3</t>
         </is>
@@ -6028,12 +6083,12 @@
       <c r="E44" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F44" s="43" t="inlineStr">
+      <c r="F44" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G44" s="38" t="inlineStr">
+      <c r="G44" s="41" t="inlineStr">
         <is>
           <t>80ca0e19-cd00-4b28-a36d-d62c1e6371e7</t>
         </is>
@@ -6061,12 +6116,12 @@
       <c r="E45" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F45" s="30" t="inlineStr">
+      <c r="F45" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G45" s="40" t="inlineStr">
+      <c r="G45" s="43" t="inlineStr">
         <is>
           <t>7f1bbf57-ff19-4729-88e6-c43e8aca6a2f</t>
         </is>
@@ -6099,7 +6154,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G46" s="38" t="inlineStr">
+      <c r="G46" s="41" t="inlineStr">
         <is>
           <t>5ce04076-8d0f-4948-8abe-c398d7e13170</t>
         </is>
@@ -6127,12 +6182,12 @@
       <c r="E47" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="F47" s="30" t="inlineStr">
+      <c r="F47" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G47" s="40" t="inlineStr">
+      <c r="G47" s="43" t="inlineStr">
         <is>
           <t>f8dd4980-8525-4726-84b2-db886a5dc006</t>
         </is>
@@ -6165,7 +6220,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G48" s="38" t="inlineStr">
+      <c r="G48" s="41" t="inlineStr">
         <is>
           <t>8aa84255-930a-4b1d-8481-990221a25cf4</t>
         </is>
@@ -6193,12 +6248,12 @@
       <c r="E49" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="F49" s="30" t="inlineStr">
+      <c r="F49" s="33" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G49" s="40" t="inlineStr">
+      <c r="G49" s="43" t="inlineStr">
         <is>
           <t>92221bb6-f4a0-43ee-bd32-675b904615c9</t>
         </is>
@@ -6231,7 +6286,7 @@
           <t>W</t>
         </is>
       </c>
-      <c r="G50" s="38" t="inlineStr">
+      <c r="G50" s="41" t="inlineStr">
         <is>
           <t>64cbdbf2-92b5-4041-9f0d-0b93b0133f46</t>
         </is>

</xml_diff>